<commit_message>
Phase 5B/5C: handling rules and Tilt (inclination) support for Panels & Fragile
Adds plan-level Handling Rules (stackable/orientation/tilt defaults with
per-item overrides) and the full Tilt/Inclination feature: signed tilt
angle within a configurable maximum, automatic packing fallback that only
inclines a panel when no valid 0-degree placement exists, manual Tilt
controls with precise OBB/SAT collision (so touching panels are valid but
real penetration is rejected), and label rendering that stays attached to
the tilted panel face. Also fixes a frontend crash where non-string
FastAPI error details (422 validation arrays) were rendered directly as
React children.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/Muestra Real.xlsx
+++ b/examples/Muestra Real.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://gcorporativo-my.sharepoint.com/personal/roberto_garcia_windowworld_com_ec/Documents/Documentos/Planificador de produccion/Proyecto de logistica/EasyCargando/examples/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="34" documentId="8_{EB1ED6BC-73C8-41C8-806D-F4F0499ECFFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{73CFCA1E-4F63-45CE-B451-4516EC57A086}"/>
+  <xr:revisionPtr revIDLastSave="36" documentId="8_{EB1ED6BC-73C8-41C8-806D-F4F0499ECFFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DA6121DC-5D29-4280-A0E2-B9C528F95039}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -995,7 +995,7 @@
   <dimension ref="A1:O110"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="6.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.42578125" customWidth="1"/>
     <col min="2" max="2" width="27.140625" customWidth="1"/>
     <col min="3" max="3" width="6.42578125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="11.140625" bestFit="1" customWidth="1"/>

</xml_diff>